<commit_message>
docs(roi): model one combined project, gate ROI to internal-only
Mixed picks are costed as a single engagement, but the ROI framing now
appears only when the project is internal-only and replaces existing
SaaS. Combining the two paths let an external product's user count
inflate hosting and maintenance, which were then charged against the
internal savings — a 2-tool project showing +346% ROI collapsed to -89%
when one web app was ticked.

Also: external user count no longer drives the tier unless an external
app is actually selected, and payback is bounded ("No payback",
"Beyond horizon") so it can never print a 320-month figure.

Outputs are marked PUBLIC or INTERNAL — raw project cost stays internal
per PRD 1 §6.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roi-calculator-config.xlsx
+++ b/docs/roi-calculator-config.xlsx
@@ -13,8 +13,7 @@
     <sheet name="Hosting" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Maintenance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Catalog" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Calc_Internal" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Calc_External" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Calc" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +75,23 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00007A33"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E1E1E"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -172,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,12 +215,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -570,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D28"/>
+  <dimension ref="A2:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -718,91 +738,79 @@
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Calc_Internal</t>
+          <t>Calc</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Live worked example — internal tools. Replace SaaS spend, see payback.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Calc_External</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Live worked example — external products. Cost vs agency benchmark.</t>
+          <t>The live model. One combined project, exactly as agreed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>WHERE THE NUMBERS CAME FROM</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>WHERE THE NUMBERS CAME FROM</t>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>• Rate tiers, consulting rate, agency benchmark: your Financial Plan 2026 sheet (Hourly Rate References / Baselines / Benchmark).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>• Rate tiers, consulting rate, agency benchmark: your Financial Plan 2026 sheet (Hourly Rate References / Baselines / Benchmark).</t>
+          <t>• Hosting bands and maintenance hours: ESTIMATES by Claude — no source. These are the least defensible numbers here; tune before launch.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>• Hosting bands and maintenance hours: ESTIMATES by Claude — no source. These are the least defensible numbers here; tune before launch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="9" t="inlineStr">
-        <is>
           <t>• Complexity weights: all default to 1.00, i.e. neutral. Raise a weight to make that app take longer.</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>AGREED DECISIONS</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>OPEN DECISIONS (see chat)</t>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>• SETTLED: public panel shows savings + % of agency. Raw project cost is INTERNAL ONLY (PRD 1 §6).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>• Does the public site show project COST, or only savings / % of agency? PRD 1 §6 says no public rates.</t>
+          <t>• SETTLED: no email gate — the result shows immediately.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>• Is the result gated behind an email capture, or shown immediately?</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>• External path has no true ROI — it is a quote estimator. Modelled here as % of agency cost.</t>
+          <t>• SETTLED: mixed picks = ONE combined project, but ROI/payback show ONLY on internal-only projects.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1521,9 +1529,13 @@
         <v>1</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Tick this and the ROI framing switches off — by design</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
@@ -1654,26 +1666,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D26"/>
+  <dimension ref="A2:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Worked example — Internal tools</t>
+          <t>The model — one combined project</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Replace SaaS you already pay for. This is the path where ROI is real.</t>
+          <t>Tick apps in Catalog. Internal and external picks become a single engagement, as agreed.</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1701,8 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -1697,526 +1711,453 @@
     <row r="6">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Employees (= users)</t>
+          <t>Employees (internal users)</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Drives tier and hosting band</t>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Drives tier and hosting if larger than external users</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Already paying for software?</t>
+          <t>Expected external users</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>1 = yes, 0 = no. If 0, there is no spend to replace.</t>
+        <v>5000</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Only asked when an external product is ticked (progressive disclosure)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Already paying for software?</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>1 = yes, 0 = no. Gates payback and ROI entirely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
           <t>Current SaaS spend ($/month)</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C9" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Ignored when the checkbox above is 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Ignored when the answer above is 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Formula in words</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Apps selected (weighted)</t>
-        </is>
-      </c>
-      <c r="C11" s="23">
-        <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"Internal",Catalog!$E$6:$E$12,1)</f>
-        <v/>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Sum of complexity weights of ticked internal apps</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="C12" s="8">
-        <f>INDEX(RateTiers!$B$6:$B$8,MATCH($C$6,RateTiers!$F$6:$F$8,1))</f>
-        <v/>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Band lookup on employee count</t>
+          <t>Internal apps (weighted)</t>
+        </is>
+      </c>
+      <c r="C12" s="23">
+        <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"Internal",Catalog!$E$6:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Ticked internal apps in Catalog</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Tier monthly rate</t>
-        </is>
-      </c>
-      <c r="C13" s="24">
-        <f>INDEX(RateTiers!$E$6:$E$8,MATCH($C$12,RateTiers!$B$6:$B$8,0))</f>
-        <v/>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>Your Low / Medium / High monthly rate</t>
+          <t>External apps (weighted)</t>
+        </is>
+      </c>
+      <c r="C13" s="23">
+        <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"External",Catalog!$E$6:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Ticked external platforms in Catalog</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Build time (months)</t>
-        </is>
-      </c>
-      <c r="C14" s="25">
-        <f>IF($C$11=0,0,Catalog!$C$17+MAX(0,$C$11-Catalog!$C$18)*Catalog!$C$19)</f>
-        <v/>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>Base + one month per weighted app beyond the base</t>
+          <t>Total apps (weighted)</t>
+        </is>
+      </c>
+      <c r="C14" s="24">
+        <f>$C$12+$C$13</f>
+        <v/>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>ONE project, so internal and external add up</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Build cost (one-off)</t>
-        </is>
-      </c>
-      <c r="C15" s="19">
-        <f>$C$13*$C$14</f>
-        <v/>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Tier monthly rate x build months</t>
+          <t>Scale driver (users)</t>
+        </is>
+      </c>
+      <c r="C15" s="25">
+        <f>MAX($C$6,IF($C$13&gt;0,$C$7,0))</f>
+        <v/>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Larger audience the system must carry. External users ignored unless an external app is ticked.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Hosting ($/month)</t>
-        </is>
-      </c>
-      <c r="C16" s="24">
-        <f>INDEX(Hosting!$D$6:$D$9,MATCH($C$6,Hosting!$C$6:$C$9,1))</f>
-        <v/>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Band lookup on employee count</t>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C16" s="8">
+        <f>INDEX(RateTiers!$B$6:$B$8,MATCH($C$15,RateTiers!$F$6:$F$8,1))</f>
+        <v/>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Band lookup on the scale driver</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Tier monthly rate</t>
+        </is>
+      </c>
+      <c r="C17" s="26">
+        <f>INDEX(RateTiers!$E$6:$E$8,MATCH($C$16,RateTiers!$B$6:$B$8,0))</f>
+        <v/>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Your Low / Medium / High monthly rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Build time (months)</t>
+        </is>
+      </c>
+      <c r="C18" s="27">
+        <f>IF($C$14=0,0,Catalog!$C$17+MAX(0,$C$14-Catalog!$C$18)*Catalog!$C$19)</f>
+        <v/>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Base + one month per weighted app beyond the base</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Hosting ($/month)</t>
+        </is>
+      </c>
+      <c r="C19" s="26">
+        <f>INDEX(Hosting!$D$6:$D$9,MATCH($C$15,Hosting!$C$6:$C$9,1))</f>
+        <v/>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Band lookup on the scale driver</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
           <t>Maintenance ($/month)</t>
         </is>
       </c>
-      <c r="C17" s="24">
-        <f>INDEX(Maintenance!$D$6:$D$8,MATCH($C$12,Maintenance!$B$6:$B$8,0))</f>
-        <v/>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C20" s="26">
+        <f>INDEX(Maintenance!$D$6:$D$8,MATCH($C$16,Maintenance!$B$6:$B$8,0))</f>
+        <v/>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Retainer hours x consulting rate</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Output — what the site shows</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Shown?</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>New monthly cost</t>
-        </is>
-      </c>
-      <c r="C20" s="26">
-        <f>$C$16+$C$17</f>
-        <v/>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Hosting + maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Monthly saving</t>
-        </is>
-      </c>
-      <c r="C21" s="26">
-        <f>IF($C$7=1,$C$8,0)-$C$20</f>
-        <v/>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Negative means the build costs more to run than today</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Payback (months)</t>
-        </is>
-      </c>
-      <c r="C22" s="27">
-        <f>IF($C$21&lt;=0,"No payback",$C$15/$C$21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>GUARD: prints text, never a negative or infinite number</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Net benefit over horizon</t>
-        </is>
-      </c>
-      <c r="C23" s="26">
-        <f>$C$21*Global!$C$5-$C$15</f>
-        <v/>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Savings across the horizon, less the build</t>
+          <t>Build cost (one-off)</t>
+        </is>
+      </c>
+      <c r="C23" s="19">
+        <f>$C$17*$C$18</f>
+        <v/>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Never rendered publicly — PRD 1 §6. For your quoting only.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
         <is>
+          <t>Agency equivalent</t>
+        </is>
+      </c>
+      <c r="C24" s="19">
+        <f>Global!$C$6*$C$18</f>
+        <v/>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Basis for the public percentage below</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>You would pay (% of agency)</t>
+        </is>
+      </c>
+      <c r="C25" s="29">
+        <f>IF($C$24&lt;=0,"n/a",$C$23/$C$24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>THE HEADLINE. Works on every path. Near 55% at High tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Build time (months)</t>
+        </is>
+      </c>
+      <c r="C26" s="31">
+        <f>$C$18</f>
+        <v/>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Always safe to show</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>New monthly cost</t>
+        </is>
+      </c>
+      <c r="C27" s="32">
+        <f>$C$19+$C$20</f>
+        <v/>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Hosting + maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Monthly saving</t>
+        </is>
+      </c>
+      <c r="C28" s="32">
+        <f>IF(AND($C$12&gt;0,$C$13=0,$C$8=1),$C$9-$C$27,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D28" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC*</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Internal-only projects. Any external pick switches this off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Payback (months)</t>
+        </is>
+      </c>
+      <c r="C29" s="31">
+        <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1),"n/a",IF($C$28&lt;=0,"No payback",IF($C$23/$C$28&gt;Global!$C$5,"Beyond horizon",$C$23/$C$28)))</f>
+        <v/>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC*</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>GUARDS: no payback, beyond horizon, or n/a — never a silly number</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Net benefit over horizon</t>
+        </is>
+      </c>
+      <c r="C30" s="32">
+        <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1),"n/a",$C$28*Global!$C$5-$C$23)</f>
+        <v/>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC*</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Savings across the horizon, less the build</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="8" t="inlineStr">
+        <is>
           <t>ROI over horizon (%)</t>
         </is>
       </c>
-      <c r="C24" s="28">
-        <f>IF($C$15&lt;=0,"n/a",$C$23/$C$15)</f>
-        <v/>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Net benefit / build cost. Meaningless without the horizon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>If 'Already paying' is 0, saving is negative and payback is text — the UI must switch to a 'new capability' framing instead of showing a broken ROI.</t>
-        </is>
-      </c>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="21" t="n"/>
+      <c r="C31" s="29">
+        <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1,$C$23&lt;=0),"n/a",$C$30/$C$23)</f>
+        <v/>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>PUBLIC*</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>ALWAYS print the horizon beside it — 346% at 36mo is 49% at 12mo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>PUBLIC* = internal-only projects that replace existing SaaS. If ANY external product is ticked, the UI drops the ROI framing and shows '% of agency' + build time instead — external scale would otherwise inflate running cost and wreck the payback maths.</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="20" t="n"/>
+      <c r="E33" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B26:D26"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A2:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Worked example — External products</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>No SaaS spend to replace, so there is no true ROI. The honest headline is cost vs an agency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Expected users</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Drives tier</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>Formula in words</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Platforms selected (weighted)</t>
-        </is>
-      </c>
-      <c r="C9" s="23">
-        <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"External",Catalog!$E$6:$E$12,1)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Sum of weights of ticked external platforms</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="C10" s="8">
-        <f>INDEX(RateTiers!$B$6:$B$8,MATCH($C$6,RateTiers!$F$6:$F$8,1))</f>
-        <v/>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Band lookup on user count</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Tier monthly rate</t>
-        </is>
-      </c>
-      <c r="C11" s="24">
-        <f>INDEX(RateTiers!$E$6:$E$8,MATCH($C$10,RateTiers!$B$6:$B$8,0))</f>
-        <v/>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Your Low / Medium / High monthly rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Build time (months)</t>
-        </is>
-      </c>
-      <c r="C12" s="25">
-        <f>IF($C$9=0,0,Catalog!$C$17+MAX(0,$C$9-Catalog!$C$18)*Catalog!$C$19)</f>
-        <v/>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Same timeline rule as internal</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Output — what the site shows</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Nalar project cost</t>
-        </is>
-      </c>
-      <c r="C15" s="26">
-        <f>$C$11*$C$12</f>
-        <v/>
-      </c>
-      <c r="D15" s="29" t="inlineStr">
-        <is>
-          <t>SENSITIVE — publishing this conflicts with PRD 1 §6</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Agency equivalent</t>
-        </is>
-      </c>
-      <c r="C16" s="26">
-        <f>Global!$C$6*$C$12</f>
-        <v/>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Benchmark monthly x the same duration</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>You would pay (% of agency)</t>
-        </is>
-      </c>
-      <c r="C17" s="28">
-        <f>IF($C$16&lt;=0,"n/a",$C$15/$C$16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>THE HEADLINE. High tier lands near 55% — the mockup's '50%'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Saving vs agency</t>
-        </is>
-      </c>
-      <c r="C18" s="26">
-        <f>$C$16-$C$15</f>
-        <v/>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Shows a big number without quoting your rate directly</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="29" t="inlineStr">
-        <is>
-          <t>'% of agency' is the one headline that works on both paths and needs no invented revenue assumptions.</t>
-        </is>
-      </c>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="21" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:E33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: adopt DEVELOPED status; simplify hosting to a formula
DEVELOPED ("built and merged, but not live") is now documented in the
PRD README and CLAUDE.md. It was already in use on the portfolio-video
doc; the convention had not caught up.

Hosting drops the four-band lookup for MAX(base, users x per-user) --
$25 + $0.30. Bands were both unsourced and discontinuous: 100 users cost
$150 and 101 cost $400, so one extra employee nearly tripled the running
cost and made payback jump for no visible reason. Two numbers to defend
instead of eight, and no AWS research needed -- hosting is the smallest
term in the comparison, so precision there does not move the headline.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roi-calculator-config.xlsx
+++ b/docs/roi-calculator-config.xlsx
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -213,10 +213,11 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -590,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D27"/>
+  <dimension ref="A2:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -707,7 +708,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Estimated AWS cost per month, banded by user count.</t>
+          <t>Base + per-user formula. Two numbers, no bands.</t>
         </is>
       </c>
     </row>
@@ -764,52 +765,60 @@
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>• Hosting bands and maintenance hours: ESTIMATES by Claude — no source. These are the least defensible numbers here; tune before launch.</t>
+          <t>• Hosting base + per-user: a deliberately simple estimate, not an AWS quote. Two numbers you can defend in a sentence.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
+          <t>• Maintenance hours: YOUR commitment, not a technical guess — how many hours a month you agree to give each tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
           <t>• Complexity weights: all default to 1.00, i.e. neutral. Raise a weight to make that app take longer.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>AGREED DECISIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>• SETTLED: public panel shows savings + % of agency. Raw project cost is INTERNAL ONLY (PRD 1 §6).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>• SETTLED: no email gate — the result shows immediately.</t>
+          <t>• SETTLED: public panel shows savings + % of agency. Raw project cost is INTERNAL ONLY (PRD 1 §6).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
+          <t>• SETTLED: no email gate — the result shows immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
           <t>• SETTLED: mixed picks = ONE combined project, but ROI/payback show ONLY on internal-only projects.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1119,136 +1128,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E11"/>
+  <dimension ref="A2:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Hosting cost (AWS estimate)</t>
+          <t>Hosting cost</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ESTIMATES — not sourced. Sorted ascending by 'From users'.</t>
+          <t>Deliberately simple: a small fixed base, plus a per-user amount. Two numbers, no bands.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Band</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>From users</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>$ / month</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>40</v>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Single small instance + managed Postgres</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Base ($/month)</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>The server exists even with one user</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>26</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>150</v>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Load-balanced, daily backups</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>101</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>400</v>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Multi-AZ, higher storage and egress</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Per user ($/month)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Scales smoothly — no cliff at a band edge</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>X-Large</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>501</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>900</v>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Scaled out; revisit properly at this size</t>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>MAX(base, users x per-user)</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>One sentence you can say out loud on a call</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Caveat: real AWS cost tracks traffic, data and concurrency — not seat count. Seats are a proxy.</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="21" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Sanity check</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Hosting / month</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Reads as</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="23">
+        <f>MAX($C$6,B13*$C$7)</f>
+        <v/>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Tiny internal tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="C14" s="23">
+        <f>MAX($C$6,B14*$C$7)</f>
+        <v/>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Typical SME headcount</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C15" s="23">
+        <f>MAX($C$6,B15*$C$7)</f>
+        <v/>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Larger team</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="23">
+        <f>MAX($C$6,B16*$C$7)</f>
+        <v/>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Small product</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C17" s="23">
+        <f>MAX($C$6,B17*$C$7)</f>
+        <v/>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Real product</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Replaced a four-band lookup table. Bands jumped $150 -&gt; $400 between 100 and 101 users; this cannot, and it is two numbers to defend instead of eight.</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1437,7 +1509,7 @@
           <t>Internal</t>
         </is>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="12" t="n">
@@ -1456,7 +1528,7 @@
           <t>Internal</t>
         </is>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="12" t="n">
@@ -1479,7 +1551,7 @@
           <t>Internal</t>
         </is>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="12" t="n">
@@ -1502,7 +1574,7 @@
           <t>Internal</t>
         </is>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="12" t="n">
@@ -1525,7 +1597,7 @@
           <t>External</t>
         </is>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="12" t="n">
@@ -1548,7 +1620,7 @@
           <t>External</t>
         </is>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="12" t="n">
@@ -1571,7 +1643,7 @@
           <t>External</t>
         </is>
       </c>
-      <c r="D12" s="22" t="n">
+      <c r="D12" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="12" t="n">
@@ -1796,7 +1868,7 @@
           <t>Internal apps (weighted)</t>
         </is>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="25">
         <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"Internal",Catalog!$E$6:$E$12,1)</f>
         <v/>
       </c>
@@ -1812,7 +1884,7 @@
           <t>External apps (weighted)</t>
         </is>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="25">
         <f>SUMIFS(Catalog!$D$6:$D$12,Catalog!$C$6:$C$12,"External",Catalog!$E$6:$E$12,1)</f>
         <v/>
       </c>
@@ -1828,7 +1900,7 @@
           <t>Total apps (weighted)</t>
         </is>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="26">
         <f>$C$12+$C$13</f>
         <v/>
       </c>
@@ -1844,7 +1916,7 @@
           <t>Scale driver (users)</t>
         </is>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="22">
         <f>MAX($C$6,IF($C$13&gt;0,$C$7,0))</f>
         <v/>
       </c>
@@ -1876,7 +1948,7 @@
           <t>Tier monthly rate</t>
         </is>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="27">
         <f>INDEX(RateTiers!$E$6:$E$8,MATCH($C$16,RateTiers!$B$6:$B$8,0))</f>
         <v/>
       </c>
@@ -1892,7 +1964,7 @@
           <t>Build time (months)</t>
         </is>
       </c>
-      <c r="C18" s="27">
+      <c r="C18" s="28">
         <f>IF($C$14=0,0,Catalog!$C$17+MAX(0,$C$14-Catalog!$C$18)*Catalog!$C$19)</f>
         <v/>
       </c>
@@ -1908,13 +1980,13 @@
           <t>Hosting ($/month)</t>
         </is>
       </c>
-      <c r="C19" s="26">
-        <f>INDEX(Hosting!$D$6:$D$9,MATCH($C$15,Hosting!$C$6:$C$9,1))</f>
+      <c r="C19" s="27">
+        <f>MAX(Hosting!$C$6,$C$15*Hosting!$C$7)</f>
         <v/>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Band lookup on the scale driver</t>
+          <t>Base + per-user, from the Hosting tab</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1996,7 @@
           <t>Maintenance ($/month)</t>
         </is>
       </c>
-      <c r="C20" s="26">
+      <c r="C20" s="27">
         <f>INDEX(Maintenance!$D$6:$D$8,MATCH($C$16,Maintenance!$B$6:$B$8,0))</f>
         <v/>
       </c>
@@ -1966,7 +2038,7 @@
         <f>$C$17*$C$18</f>
         <v/>
       </c>
-      <c r="D23" s="28" t="inlineStr">
+      <c r="D23" s="29" t="inlineStr">
         <is>
           <t>INTERNAL</t>
         </is>
@@ -1987,7 +2059,7 @@
         <f>Global!$C$6*$C$18</f>
         <v/>
       </c>
-      <c r="D24" s="28" t="inlineStr">
+      <c r="D24" s="29" t="inlineStr">
         <is>
           <t>INTERNAL</t>
         </is>
@@ -2004,11 +2076,11 @@
           <t>You would pay (% of agency)</t>
         </is>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="30">
         <f>IF($C$24&lt;=0,"n/a",$C$23/$C$24)</f>
         <v/>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="31" t="inlineStr">
         <is>
           <t>PUBLIC</t>
         </is>
@@ -2025,11 +2097,11 @@
           <t>Build time (months)</t>
         </is>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="32">
         <f>$C$18</f>
         <v/>
       </c>
-      <c r="D26" s="30" t="inlineStr">
+      <c r="D26" s="31" t="inlineStr">
         <is>
           <t>PUBLIC</t>
         </is>
@@ -2046,11 +2118,11 @@
           <t>New monthly cost</t>
         </is>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="33">
         <f>$C$19+$C$20</f>
         <v/>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>PUBLIC</t>
         </is>
@@ -2067,11 +2139,11 @@
           <t>Monthly saving</t>
         </is>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="33">
         <f>IF(AND($C$12&gt;0,$C$13=0,$C$8=1),$C$9-$C$27,"n/a")</f>
         <v/>
       </c>
-      <c r="D28" s="30" t="inlineStr">
+      <c r="D28" s="31" t="inlineStr">
         <is>
           <t>PUBLIC*</t>
         </is>
@@ -2088,11 +2160,11 @@
           <t>Payback (months)</t>
         </is>
       </c>
-      <c r="C29" s="31">
+      <c r="C29" s="32">
         <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1),"n/a",IF($C$28&lt;=0,"No payback",IF($C$23/$C$28&gt;Global!$C$5,"Beyond horizon",$C$23/$C$28)))</f>
         <v/>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D29" s="31" t="inlineStr">
         <is>
           <t>PUBLIC*</t>
         </is>
@@ -2109,11 +2181,11 @@
           <t>Net benefit over horizon</t>
         </is>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="33">
         <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1),"n/a",$C$28*Global!$C$5-$C$23)</f>
         <v/>
       </c>
-      <c r="D30" s="30" t="inlineStr">
+      <c r="D30" s="31" t="inlineStr">
         <is>
           <t>PUBLIC*</t>
         </is>
@@ -2130,11 +2202,11 @@
           <t>ROI over horizon (%)</t>
         </is>
       </c>
-      <c r="C31" s="29">
+      <c r="C31" s="30">
         <f>IF(OR($C$12=0,$C$13&gt;0,$C$8&lt;&gt;1,$C$23&lt;=0),"n/a",$C$30/$C$23)</f>
         <v/>
       </c>
-      <c r="D31" s="30" t="inlineStr">
+      <c r="D31" s="31" t="inlineStr">
         <is>
           <t>PUBLIC*</t>
         </is>
@@ -2146,7 +2218,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="33" t="inlineStr">
+      <c r="B33" s="34" t="inlineStr">
         <is>
           <t>PUBLIC* = internal-only projects that replace existing SaaS. If ANY external product is ticked, the UI drops the ROI framing and shows '% of agency' + build time instead — external scale would otherwise inflate running cost and wreck the payback maths.</t>
         </is>

</xml_diff>